<commit_message>
Table S4: add FaIR_comb_unB as an individual reference block (1850-1900)
fut_fair_worker.py (generated by make_oscar_worker.py from fut2_fix_worker.py) scores FaIR_comb_unB, the method
with the largest CSCM stacking weight, as an individual reference under the same leave-one-out protocol as
EBMKF_ta4 / GWI_tot_CGWL (2000-2089 window, 1850-1900 datum). 270 member results are in
results/FaIR_comb_unB_individual_b1900/. check_and_aggregate.py takes them as an optional fourth argument and
appends one block to table-S4-for-docs and table-S4-individual-references.csv. A fresh aggregation reproduces
the output_b1900 tables byte for byte.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fut_LOO/output_b1900/table-S4-for-docs.xlsx
+++ b/fut_LOO/output_b1900/table-S4-for-docs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2776,6 +2776,294 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FaIR_comb_unB</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>MPI-ESM1-2-LR SSP3-7.0</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>20.9%</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>43.1%</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>89.2%</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0.648</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>0.419</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>0.0612</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>0.0499</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>FaIR_comb_unB</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>MPI-ESM1-2-LR SSP2-4.5</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>26.7%</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>52.4%</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>95.4%</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0.688</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>0.556</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>0.0452</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>0.0408</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>FaIR_comb_unB</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MPI-ESM1-2-LR SSP1-2.6</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>9.7%</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>45.0%</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>0.801</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>0.814</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>1.360</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>0.0576</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>0.0575</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>FaIR_comb_unB</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NorESM RCP4.5 (constant volcanic)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>29.0%</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>55.1%</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>91.6%</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>0.762</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>0.695</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>0.0469</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>0.0453</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>FaIR_comb_unB</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NorESM RCP4.5 (volcanic)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>20.2%</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>38.9%</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>77.2%</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>0.834</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>0.843</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>1.150</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>0.0662</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>0.0677</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>